<commit_message>
Correction du waterfall du drill : le graphe ne s'affichait pas
Les series du waterfall etaient dans les colonnes K:O que j'avais masquees.
Excel ecrit plotVisOnly=1 par defaut et ne trace pas les cellules masquees :
le graphe s'ouvrait vide. Ajout de visible_cells_only=False.

Deux corrections de lisibilite au passage :
- axe resserre de 80-150 k EUR a 90-145 k EUR : a l'ancienne echelle la barre
  de l'effet cout variable (1 364 EUR) faisait moins de trois pixels et son
  etiquette ne tenait pas.
- titre raccourci en "EBITDA TUNON_PAR - 2025 -> 2026" : l'ancien tenait sur
  trois lignes et ecrasait la zone de trace ; le message reste dans l'encadre
  sous le graphe.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/DRILL_SIMULATION.xlsx
+++ b/eduservices/DRILL_SIMULATION.xlsx
@@ -748,7 +748,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Pourquoi l'EBITDA de TUNON_PAR recule de 10 500 € : la croissance existe, les coûts fixes la mangent</a:t>
+              <a:t>EBITDA TUNON_PAR  ·  2025 → 2026</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -899,8 +899,8 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="150000"/>
-          <min val="80000"/>
+          <max val="145000"/>
+          <min val="90000"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -912,7 +912,7 @@
         <majorUnit val="10000"/>
       </valAx>
     </plotArea>
-    <plotVisOnly val="1"/>
+    <plotVisOnly val="0"/>
     <dispBlanksAs val="gap"/>
   </chart>
 </chartSpace>

</xml_diff>